<commit_message>
HR Excel Data Analysis
</commit_message>
<xml_diff>
--- a/HR_Capstone_Completed_Kaothar_Owolabi.xlsx
+++ b/HR_Capstone_Completed_Kaothar_Owolabi.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{E0169833-4E99-4BC8-AD5C-297FEA1FB4DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BFDBD64-7A45-4EC2-9567-10AE33CC584E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Employee_Data" sheetId="4" r:id="rId1"/>
@@ -1284,22 +1284,16 @@
   </cellStyles>
   <dxfs count="19">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="167" formatCode="[$₦-466]\ #,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="[$₦-466]\ #,##0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="[$₦-466]\ #,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="[$₦-466]\ #,##0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="167" formatCode="[$₦-466]\ #,##0"/>
@@ -1318,6 +1312,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -11160,643 +11160,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CB9A93F9-6FD6-48A0-8F2E-4F3900894424}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" rowHeaderCaption="Employment Status">
-  <location ref="A15:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="17">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="148">
-        <item x="35"/>
-        <item x="72"/>
-        <item x="93"/>
-        <item x="61"/>
-        <item x="30"/>
-        <item x="137"/>
-        <item x="69"/>
-        <item x="29"/>
-        <item x="134"/>
-        <item x="90"/>
-        <item x="98"/>
-        <item x="78"/>
-        <item x="16"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="145"/>
-        <item x="125"/>
-        <item x="44"/>
-        <item x="102"/>
-        <item x="143"/>
-        <item x="23"/>
-        <item x="19"/>
-        <item x="50"/>
-        <item x="111"/>
-        <item x="73"/>
-        <item x="64"/>
-        <item x="105"/>
-        <item x="107"/>
-        <item x="47"/>
-        <item x="75"/>
-        <item x="34"/>
-        <item x="133"/>
-        <item x="65"/>
-        <item x="62"/>
-        <item x="87"/>
-        <item x="60"/>
-        <item x="17"/>
-        <item x="20"/>
-        <item x="136"/>
-        <item x="127"/>
-        <item x="118"/>
-        <item x="39"/>
-        <item x="68"/>
-        <item x="113"/>
-        <item x="130"/>
-        <item x="0"/>
-        <item x="100"/>
-        <item x="70"/>
-        <item x="88"/>
-        <item x="40"/>
-        <item x="122"/>
-        <item x="94"/>
-        <item x="28"/>
-        <item x="18"/>
-        <item x="135"/>
-        <item x="91"/>
-        <item x="8"/>
-        <item x="56"/>
-        <item x="124"/>
-        <item x="123"/>
-        <item x="131"/>
-        <item x="79"/>
-        <item x="92"/>
-        <item x="52"/>
-        <item x="106"/>
-        <item x="42"/>
-        <item x="74"/>
-        <item x="66"/>
-        <item x="77"/>
-        <item x="138"/>
-        <item x="89"/>
-        <item x="51"/>
-        <item x="97"/>
-        <item x="43"/>
-        <item x="26"/>
-        <item x="32"/>
-        <item x="45"/>
-        <item x="86"/>
-        <item x="141"/>
-        <item x="14"/>
-        <item x="5"/>
-        <item x="101"/>
-        <item x="139"/>
-        <item x="10"/>
-        <item x="38"/>
-        <item x="59"/>
-        <item x="114"/>
-        <item x="48"/>
-        <item x="109"/>
-        <item x="13"/>
-        <item x="41"/>
-        <item x="96"/>
-        <item x="84"/>
-        <item x="7"/>
-        <item x="120"/>
-        <item x="55"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="21"/>
-        <item x="12"/>
-        <item x="132"/>
-        <item x="82"/>
-        <item x="76"/>
-        <item x="104"/>
-        <item x="67"/>
-        <item x="108"/>
-        <item x="85"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="117"/>
-        <item x="116"/>
-        <item x="33"/>
-        <item x="121"/>
-        <item x="49"/>
-        <item x="36"/>
-        <item x="129"/>
-        <item x="126"/>
-        <item x="112"/>
-        <item x="110"/>
-        <item x="144"/>
-        <item x="24"/>
-        <item x="37"/>
-        <item x="81"/>
-        <item x="27"/>
-        <item x="1"/>
-        <item x="71"/>
-        <item x="63"/>
-        <item x="146"/>
-        <item x="22"/>
-        <item x="80"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="119"/>
-        <item x="83"/>
-        <item x="115"/>
-        <item x="142"/>
-        <item x="54"/>
-        <item x="140"/>
-        <item x="25"/>
-        <item x="15"/>
-        <item x="99"/>
-        <item x="31"/>
-        <item x="58"/>
-        <item x="128"/>
-        <item x="57"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="2" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="12">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="10"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average Performance Score" fld="9" subtotal="average" baseField="10" baseItem="0"/>
-  </dataFields>
-  <formats count="4">
-    <format dxfId="3">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="10" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="2">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="10" count="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="1">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="10" count="1">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="0">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="5">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="9">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="9" format="10">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="10" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9EC9E3F-503E-4ED3-BE09-02423CB7D4D3}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:A4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="17">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="148">
-        <item x="35"/>
-        <item x="72"/>
-        <item x="93"/>
-        <item x="61"/>
-        <item x="30"/>
-        <item x="137"/>
-        <item x="69"/>
-        <item x="29"/>
-        <item x="134"/>
-        <item x="90"/>
-        <item x="98"/>
-        <item x="78"/>
-        <item x="16"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="145"/>
-        <item x="125"/>
-        <item x="44"/>
-        <item x="102"/>
-        <item x="143"/>
-        <item x="23"/>
-        <item x="19"/>
-        <item x="50"/>
-        <item x="111"/>
-        <item x="73"/>
-        <item x="64"/>
-        <item x="105"/>
-        <item x="107"/>
-        <item x="47"/>
-        <item x="75"/>
-        <item x="34"/>
-        <item x="133"/>
-        <item x="65"/>
-        <item x="62"/>
-        <item x="87"/>
-        <item x="60"/>
-        <item x="17"/>
-        <item x="20"/>
-        <item x="136"/>
-        <item x="127"/>
-        <item x="118"/>
-        <item x="39"/>
-        <item x="68"/>
-        <item x="113"/>
-        <item x="130"/>
-        <item x="0"/>
-        <item x="100"/>
-        <item x="70"/>
-        <item x="88"/>
-        <item x="40"/>
-        <item x="122"/>
-        <item x="94"/>
-        <item x="28"/>
-        <item x="18"/>
-        <item x="135"/>
-        <item x="91"/>
-        <item x="8"/>
-        <item x="56"/>
-        <item x="124"/>
-        <item x="123"/>
-        <item x="131"/>
-        <item x="79"/>
-        <item x="92"/>
-        <item x="52"/>
-        <item x="106"/>
-        <item x="42"/>
-        <item x="74"/>
-        <item x="66"/>
-        <item x="77"/>
-        <item x="138"/>
-        <item x="89"/>
-        <item x="51"/>
-        <item x="97"/>
-        <item x="43"/>
-        <item x="26"/>
-        <item x="32"/>
-        <item x="45"/>
-        <item x="86"/>
-        <item x="141"/>
-        <item x="14"/>
-        <item x="5"/>
-        <item x="101"/>
-        <item x="139"/>
-        <item x="10"/>
-        <item x="38"/>
-        <item x="59"/>
-        <item x="114"/>
-        <item x="48"/>
-        <item x="109"/>
-        <item x="13"/>
-        <item x="41"/>
-        <item x="96"/>
-        <item x="84"/>
-        <item x="7"/>
-        <item x="120"/>
-        <item x="55"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="21"/>
-        <item x="12"/>
-        <item x="132"/>
-        <item x="82"/>
-        <item x="76"/>
-        <item x="104"/>
-        <item x="67"/>
-        <item x="108"/>
-        <item x="85"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="117"/>
-        <item x="116"/>
-        <item x="33"/>
-        <item x="121"/>
-        <item x="49"/>
-        <item x="36"/>
-        <item x="129"/>
-        <item x="126"/>
-        <item x="112"/>
-        <item x="110"/>
-        <item x="144"/>
-        <item x="24"/>
-        <item x="37"/>
-        <item x="81"/>
-        <item x="27"/>
-        <item x="1"/>
-        <item x="71"/>
-        <item x="63"/>
-        <item x="146"/>
-        <item x="22"/>
-        <item x="80"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="119"/>
-        <item x="83"/>
-        <item x="115"/>
-        <item x="142"/>
-        <item x="54"/>
-        <item x="140"/>
-        <item x="25"/>
-        <item x="15"/>
-        <item x="99"/>
-        <item x="31"/>
-        <item x="58"/>
-        <item x="128"/>
-        <item x="57"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="2" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="12">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Total Employee" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B739BF9A-5FC7-42A1-9853-4FCDDD0AC675}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
   <location ref="D3:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
@@ -12071,10 +11434,10 @@
     <dataField name="Average Salary" fld="8" subtotal="average" baseField="5" baseItem="0" numFmtId="166"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="5">
+    <format dxfId="1">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="0">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
@@ -12094,7 +11457,321 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B3D8AE2-6A64-4099-9458-D506A3DD7E3C}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="22" rowHeaderCaption="Performance Band">
+  <location ref="E26:F33" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="148">
+        <item x="35"/>
+        <item x="72"/>
+        <item x="93"/>
+        <item x="61"/>
+        <item x="30"/>
+        <item x="137"/>
+        <item x="69"/>
+        <item x="29"/>
+        <item x="134"/>
+        <item x="90"/>
+        <item x="98"/>
+        <item x="78"/>
+        <item x="16"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="145"/>
+        <item x="125"/>
+        <item x="44"/>
+        <item x="102"/>
+        <item x="143"/>
+        <item x="23"/>
+        <item x="19"/>
+        <item x="50"/>
+        <item x="111"/>
+        <item x="73"/>
+        <item x="64"/>
+        <item x="105"/>
+        <item x="107"/>
+        <item x="47"/>
+        <item x="75"/>
+        <item x="34"/>
+        <item x="133"/>
+        <item x="65"/>
+        <item x="62"/>
+        <item x="87"/>
+        <item x="60"/>
+        <item x="17"/>
+        <item x="20"/>
+        <item x="136"/>
+        <item x="127"/>
+        <item x="118"/>
+        <item x="39"/>
+        <item x="68"/>
+        <item x="113"/>
+        <item x="130"/>
+        <item x="0"/>
+        <item x="100"/>
+        <item x="70"/>
+        <item x="88"/>
+        <item x="40"/>
+        <item x="122"/>
+        <item x="94"/>
+        <item x="28"/>
+        <item x="18"/>
+        <item x="135"/>
+        <item x="91"/>
+        <item x="8"/>
+        <item x="56"/>
+        <item x="124"/>
+        <item x="123"/>
+        <item x="131"/>
+        <item x="79"/>
+        <item x="92"/>
+        <item x="52"/>
+        <item x="106"/>
+        <item x="42"/>
+        <item x="74"/>
+        <item x="66"/>
+        <item x="77"/>
+        <item x="138"/>
+        <item x="89"/>
+        <item x="51"/>
+        <item x="97"/>
+        <item x="43"/>
+        <item x="26"/>
+        <item x="32"/>
+        <item x="45"/>
+        <item x="86"/>
+        <item x="141"/>
+        <item x="14"/>
+        <item x="5"/>
+        <item x="101"/>
+        <item x="139"/>
+        <item x="10"/>
+        <item x="38"/>
+        <item x="59"/>
+        <item x="114"/>
+        <item x="48"/>
+        <item x="109"/>
+        <item x="13"/>
+        <item x="41"/>
+        <item x="96"/>
+        <item x="84"/>
+        <item x="7"/>
+        <item x="120"/>
+        <item x="55"/>
+        <item x="53"/>
+        <item x="103"/>
+        <item x="21"/>
+        <item x="12"/>
+        <item x="132"/>
+        <item x="82"/>
+        <item x="76"/>
+        <item x="104"/>
+        <item x="67"/>
+        <item x="108"/>
+        <item x="85"/>
+        <item x="46"/>
+        <item x="95"/>
+        <item x="117"/>
+        <item x="116"/>
+        <item x="33"/>
+        <item x="121"/>
+        <item x="49"/>
+        <item x="36"/>
+        <item x="129"/>
+        <item x="126"/>
+        <item x="112"/>
+        <item x="110"/>
+        <item x="144"/>
+        <item x="24"/>
+        <item x="37"/>
+        <item x="81"/>
+        <item x="27"/>
+        <item x="1"/>
+        <item x="71"/>
+        <item x="63"/>
+        <item x="146"/>
+        <item x="22"/>
+        <item x="80"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="119"/>
+        <item x="83"/>
+        <item x="115"/>
+        <item x="142"/>
+        <item x="54"/>
+        <item x="140"/>
+        <item x="25"/>
+        <item x="15"/>
+        <item x="99"/>
+        <item x="31"/>
+        <item x="58"/>
+        <item x="128"/>
+        <item x="57"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="2" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Perf_Score" fld="9" subtotal="average" baseField="5" baseItem="0"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="19" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{38A041E8-98EA-473D-A2C0-7082AD093121}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Performance Band">
   <location ref="E15:F21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
@@ -12375,7 +12052,7 @@
     <dataField name="Bonus Payout" fld="13" baseField="11" baseItem="0" numFmtId="167"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="6">
+    <format dxfId="4">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -12402,7 +12079,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{74F40968-11FB-48F2-848F-A68D40BE9B3E}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18" rowHeaderCaption="Hire Year">
   <location ref="D40:E50" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
@@ -12686,10 +12363,10 @@
     <dataField name="Average Perf_Score" fld="9" subtotal="average" baseField="16" baseItem="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="8">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -12705,7 +12382,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD033A26-7B2B-48E7-A93A-4E54A38FB54A}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19" rowHeaderCaption="Performance Band">
   <location ref="A25:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
@@ -12989,13 +12666,13 @@
     <dataField name="Count of Emp ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="11">
+    <format dxfId="9">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="7">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -13031,7 +12708,644 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CB9A93F9-6FD6-48A0-8F2E-4F3900894424}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" rowHeaderCaption="Employment Status">
+  <location ref="A15:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="148">
+        <item x="35"/>
+        <item x="72"/>
+        <item x="93"/>
+        <item x="61"/>
+        <item x="30"/>
+        <item x="137"/>
+        <item x="69"/>
+        <item x="29"/>
+        <item x="134"/>
+        <item x="90"/>
+        <item x="98"/>
+        <item x="78"/>
+        <item x="16"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="145"/>
+        <item x="125"/>
+        <item x="44"/>
+        <item x="102"/>
+        <item x="143"/>
+        <item x="23"/>
+        <item x="19"/>
+        <item x="50"/>
+        <item x="111"/>
+        <item x="73"/>
+        <item x="64"/>
+        <item x="105"/>
+        <item x="107"/>
+        <item x="47"/>
+        <item x="75"/>
+        <item x="34"/>
+        <item x="133"/>
+        <item x="65"/>
+        <item x="62"/>
+        <item x="87"/>
+        <item x="60"/>
+        <item x="17"/>
+        <item x="20"/>
+        <item x="136"/>
+        <item x="127"/>
+        <item x="118"/>
+        <item x="39"/>
+        <item x="68"/>
+        <item x="113"/>
+        <item x="130"/>
+        <item x="0"/>
+        <item x="100"/>
+        <item x="70"/>
+        <item x="88"/>
+        <item x="40"/>
+        <item x="122"/>
+        <item x="94"/>
+        <item x="28"/>
+        <item x="18"/>
+        <item x="135"/>
+        <item x="91"/>
+        <item x="8"/>
+        <item x="56"/>
+        <item x="124"/>
+        <item x="123"/>
+        <item x="131"/>
+        <item x="79"/>
+        <item x="92"/>
+        <item x="52"/>
+        <item x="106"/>
+        <item x="42"/>
+        <item x="74"/>
+        <item x="66"/>
+        <item x="77"/>
+        <item x="138"/>
+        <item x="89"/>
+        <item x="51"/>
+        <item x="97"/>
+        <item x="43"/>
+        <item x="26"/>
+        <item x="32"/>
+        <item x="45"/>
+        <item x="86"/>
+        <item x="141"/>
+        <item x="14"/>
+        <item x="5"/>
+        <item x="101"/>
+        <item x="139"/>
+        <item x="10"/>
+        <item x="38"/>
+        <item x="59"/>
+        <item x="114"/>
+        <item x="48"/>
+        <item x="109"/>
+        <item x="13"/>
+        <item x="41"/>
+        <item x="96"/>
+        <item x="84"/>
+        <item x="7"/>
+        <item x="120"/>
+        <item x="55"/>
+        <item x="53"/>
+        <item x="103"/>
+        <item x="21"/>
+        <item x="12"/>
+        <item x="132"/>
+        <item x="82"/>
+        <item x="76"/>
+        <item x="104"/>
+        <item x="67"/>
+        <item x="108"/>
+        <item x="85"/>
+        <item x="46"/>
+        <item x="95"/>
+        <item x="117"/>
+        <item x="116"/>
+        <item x="33"/>
+        <item x="121"/>
+        <item x="49"/>
+        <item x="36"/>
+        <item x="129"/>
+        <item x="126"/>
+        <item x="112"/>
+        <item x="110"/>
+        <item x="144"/>
+        <item x="24"/>
+        <item x="37"/>
+        <item x="81"/>
+        <item x="27"/>
+        <item x="1"/>
+        <item x="71"/>
+        <item x="63"/>
+        <item x="146"/>
+        <item x="22"/>
+        <item x="80"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="119"/>
+        <item x="83"/>
+        <item x="115"/>
+        <item x="142"/>
+        <item x="54"/>
+        <item x="140"/>
+        <item x="25"/>
+        <item x="15"/>
+        <item x="99"/>
+        <item x="31"/>
+        <item x="58"/>
+        <item x="128"/>
+        <item x="57"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="2" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average Performance Score" fld="9" subtotal="average" baseField="10" baseItem="0"/>
+  </dataFields>
+  <formats count="4">
+    <format dxfId="13">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="10" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="10" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="11">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="10" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="5">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="9" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9EC9E3F-503E-4ED3-BE09-02423CB7D4D3}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:A4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="17">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="148">
+        <item x="35"/>
+        <item x="72"/>
+        <item x="93"/>
+        <item x="61"/>
+        <item x="30"/>
+        <item x="137"/>
+        <item x="69"/>
+        <item x="29"/>
+        <item x="134"/>
+        <item x="90"/>
+        <item x="98"/>
+        <item x="78"/>
+        <item x="16"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="145"/>
+        <item x="125"/>
+        <item x="44"/>
+        <item x="102"/>
+        <item x="143"/>
+        <item x="23"/>
+        <item x="19"/>
+        <item x="50"/>
+        <item x="111"/>
+        <item x="73"/>
+        <item x="64"/>
+        <item x="105"/>
+        <item x="107"/>
+        <item x="47"/>
+        <item x="75"/>
+        <item x="34"/>
+        <item x="133"/>
+        <item x="65"/>
+        <item x="62"/>
+        <item x="87"/>
+        <item x="60"/>
+        <item x="17"/>
+        <item x="20"/>
+        <item x="136"/>
+        <item x="127"/>
+        <item x="118"/>
+        <item x="39"/>
+        <item x="68"/>
+        <item x="113"/>
+        <item x="130"/>
+        <item x="0"/>
+        <item x="100"/>
+        <item x="70"/>
+        <item x="88"/>
+        <item x="40"/>
+        <item x="122"/>
+        <item x="94"/>
+        <item x="28"/>
+        <item x="18"/>
+        <item x="135"/>
+        <item x="91"/>
+        <item x="8"/>
+        <item x="56"/>
+        <item x="124"/>
+        <item x="123"/>
+        <item x="131"/>
+        <item x="79"/>
+        <item x="92"/>
+        <item x="52"/>
+        <item x="106"/>
+        <item x="42"/>
+        <item x="74"/>
+        <item x="66"/>
+        <item x="77"/>
+        <item x="138"/>
+        <item x="89"/>
+        <item x="51"/>
+        <item x="97"/>
+        <item x="43"/>
+        <item x="26"/>
+        <item x="32"/>
+        <item x="45"/>
+        <item x="86"/>
+        <item x="141"/>
+        <item x="14"/>
+        <item x="5"/>
+        <item x="101"/>
+        <item x="139"/>
+        <item x="10"/>
+        <item x="38"/>
+        <item x="59"/>
+        <item x="114"/>
+        <item x="48"/>
+        <item x="109"/>
+        <item x="13"/>
+        <item x="41"/>
+        <item x="96"/>
+        <item x="84"/>
+        <item x="7"/>
+        <item x="120"/>
+        <item x="55"/>
+        <item x="53"/>
+        <item x="103"/>
+        <item x="21"/>
+        <item x="12"/>
+        <item x="132"/>
+        <item x="82"/>
+        <item x="76"/>
+        <item x="104"/>
+        <item x="67"/>
+        <item x="108"/>
+        <item x="85"/>
+        <item x="46"/>
+        <item x="95"/>
+        <item x="117"/>
+        <item x="116"/>
+        <item x="33"/>
+        <item x="121"/>
+        <item x="49"/>
+        <item x="36"/>
+        <item x="129"/>
+        <item x="126"/>
+        <item x="112"/>
+        <item x="110"/>
+        <item x="144"/>
+        <item x="24"/>
+        <item x="37"/>
+        <item x="81"/>
+        <item x="27"/>
+        <item x="1"/>
+        <item x="71"/>
+        <item x="63"/>
+        <item x="146"/>
+        <item x="22"/>
+        <item x="80"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="119"/>
+        <item x="83"/>
+        <item x="115"/>
+        <item x="142"/>
+        <item x="54"/>
+        <item x="140"/>
+        <item x="25"/>
+        <item x="15"/>
+        <item x="99"/>
+        <item x="31"/>
+        <item x="58"/>
+        <item x="128"/>
+        <item x="57"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="2" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Total Employee" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F86EDFF5-6463-43C1-906C-8E9E3325382B}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Departments">
   <location ref="I3:J26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
@@ -13369,320 +13683,6 @@
       </extLst>
     </dataField>
   </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B3D8AE2-6A64-4099-9458-D506A3DD7E3C}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="22" rowHeaderCaption="Performance Band">
-  <location ref="E26:F33" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="17">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="148">
-        <item x="35"/>
-        <item x="72"/>
-        <item x="93"/>
-        <item x="61"/>
-        <item x="30"/>
-        <item x="137"/>
-        <item x="69"/>
-        <item x="29"/>
-        <item x="134"/>
-        <item x="90"/>
-        <item x="98"/>
-        <item x="78"/>
-        <item x="16"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="145"/>
-        <item x="125"/>
-        <item x="44"/>
-        <item x="102"/>
-        <item x="143"/>
-        <item x="23"/>
-        <item x="19"/>
-        <item x="50"/>
-        <item x="111"/>
-        <item x="73"/>
-        <item x="64"/>
-        <item x="105"/>
-        <item x="107"/>
-        <item x="47"/>
-        <item x="75"/>
-        <item x="34"/>
-        <item x="133"/>
-        <item x="65"/>
-        <item x="62"/>
-        <item x="87"/>
-        <item x="60"/>
-        <item x="17"/>
-        <item x="20"/>
-        <item x="136"/>
-        <item x="127"/>
-        <item x="118"/>
-        <item x="39"/>
-        <item x="68"/>
-        <item x="113"/>
-        <item x="130"/>
-        <item x="0"/>
-        <item x="100"/>
-        <item x="70"/>
-        <item x="88"/>
-        <item x="40"/>
-        <item x="122"/>
-        <item x="94"/>
-        <item x="28"/>
-        <item x="18"/>
-        <item x="135"/>
-        <item x="91"/>
-        <item x="8"/>
-        <item x="56"/>
-        <item x="124"/>
-        <item x="123"/>
-        <item x="131"/>
-        <item x="79"/>
-        <item x="92"/>
-        <item x="52"/>
-        <item x="106"/>
-        <item x="42"/>
-        <item x="74"/>
-        <item x="66"/>
-        <item x="77"/>
-        <item x="138"/>
-        <item x="89"/>
-        <item x="51"/>
-        <item x="97"/>
-        <item x="43"/>
-        <item x="26"/>
-        <item x="32"/>
-        <item x="45"/>
-        <item x="86"/>
-        <item x="141"/>
-        <item x="14"/>
-        <item x="5"/>
-        <item x="101"/>
-        <item x="139"/>
-        <item x="10"/>
-        <item x="38"/>
-        <item x="59"/>
-        <item x="114"/>
-        <item x="48"/>
-        <item x="109"/>
-        <item x="13"/>
-        <item x="41"/>
-        <item x="96"/>
-        <item x="84"/>
-        <item x="7"/>
-        <item x="120"/>
-        <item x="55"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="21"/>
-        <item x="12"/>
-        <item x="132"/>
-        <item x="82"/>
-        <item x="76"/>
-        <item x="104"/>
-        <item x="67"/>
-        <item x="108"/>
-        <item x="85"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="117"/>
-        <item x="116"/>
-        <item x="33"/>
-        <item x="121"/>
-        <item x="49"/>
-        <item x="36"/>
-        <item x="129"/>
-        <item x="126"/>
-        <item x="112"/>
-        <item x="110"/>
-        <item x="144"/>
-        <item x="24"/>
-        <item x="37"/>
-        <item x="81"/>
-        <item x="27"/>
-        <item x="1"/>
-        <item x="71"/>
-        <item x="63"/>
-        <item x="146"/>
-        <item x="22"/>
-        <item x="80"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="119"/>
-        <item x="83"/>
-        <item x="115"/>
-        <item x="142"/>
-        <item x="54"/>
-        <item x="140"/>
-        <item x="25"/>
-        <item x="15"/>
-        <item x="99"/>
-        <item x="31"/>
-        <item x="58"/>
-        <item x="128"/>
-        <item x="57"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="2" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="12">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Perf_Score" fld="9" subtotal="average" baseField="5" baseItem="0"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="13">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="12">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="19" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">

</xml_diff>